<commit_message>
update with flgith_dispersal information
</commit_message>
<xml_diff>
--- a/data/topID feeding guild.xlsx
+++ b/data/topID feeding guild.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osawe\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osawe\Documents\Git\cc-urbanization\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D49DB343-5858-462D-91F0-62FFFBF6D187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78ED513-8519-4154-84DF-283C792FB51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{49CD93DB-F6D1-459A-A250-6E9A2941DB32}"/>
+    <workbookView xWindow="22335" yWindow="3480" windowWidth="23865" windowHeight="17655" xr2:uid="{49CD93DB-F6D1-459A-A250-6E9A2941DB32}"/>
   </bookViews>
   <sheets>
     <sheet name="topID" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="88">
   <si>
     <t>Rank</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>Scavangers</t>
+  </si>
+  <si>
+    <t>Dispersal_Flight</t>
   </si>
 </sst>
 </file>
@@ -823,10 +826,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1146,13 +1145,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63FA7C4E-3E85-46B7-BDCD-623AD9316B3B}">
-  <dimension ref="A1:G69"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H69"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1174,8 +1174,11 @@
       <c r="G1" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1197,8 +1200,11 @@
       <c r="G2">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1220,8 +1226,11 @@
       <c r="G3">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1243,8 +1252,11 @@
       <c r="G4">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1266,8 +1278,11 @@
       <c r="G5">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -1289,8 +1304,11 @@
       <c r="G6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -1312,8 +1330,11 @@
       <c r="G7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1335,8 +1356,11 @@
       <c r="G8">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1358,8 +1382,11 @@
       <c r="G9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1381,8 +1408,11 @@
       <c r="G10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1404,8 +1434,11 @@
       <c r="G11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1427,8 +1460,11 @@
       <c r="G12">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1450,8 +1486,11 @@
       <c r="G13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1473,8 +1512,11 @@
       <c r="G14">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H14">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>3</v>
       </c>
@@ -1496,8 +1538,11 @@
       <c r="G15">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H15">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>3</v>
       </c>
@@ -1519,8 +1564,11 @@
       <c r="G16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H16">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>3</v>
       </c>
@@ -1542,8 +1590,11 @@
       <c r="G17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H17">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -1565,8 +1616,11 @@
       <c r="G18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H18">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>3</v>
       </c>
@@ -1588,8 +1642,11 @@
       <c r="G19">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H19">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -1611,8 +1668,11 @@
       <c r="G20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H20">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>3</v>
       </c>
@@ -1634,8 +1694,11 @@
       <c r="G21">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H21">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>3</v>
       </c>
@@ -1657,8 +1720,11 @@
       <c r="G22">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H22">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>3</v>
       </c>
@@ -1680,8 +1746,11 @@
       <c r="G23">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H23">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>3</v>
       </c>
@@ -1703,8 +1772,11 @@
       <c r="G24">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H24">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -1726,8 +1798,11 @@
       <c r="G25">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H25">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>3</v>
       </c>
@@ -1749,8 +1824,11 @@
       <c r="G26">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H26">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1772,8 +1850,11 @@
       <c r="G27">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H27">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>3</v>
       </c>
@@ -1795,8 +1876,11 @@
       <c r="G28">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H28">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>3</v>
       </c>
@@ -1818,8 +1902,11 @@
       <c r="G29">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H29">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>3</v>
       </c>
@@ -1841,8 +1928,11 @@
       <c r="G30">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H30">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>3</v>
       </c>
@@ -1864,8 +1954,11 @@
       <c r="G31">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H31">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -1887,8 +1980,11 @@
       <c r="G32">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H32">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>40</v>
       </c>
@@ -1910,8 +2006,11 @@
       <c r="G33">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H33">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>3</v>
       </c>
@@ -1933,8 +2032,11 @@
       <c r="G34">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H34">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>3</v>
       </c>
@@ -1956,8 +2058,11 @@
       <c r="G35">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H35">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>3</v>
       </c>
@@ -1979,8 +2084,11 @@
       <c r="G36">
         <v>0.8</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H36">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>3</v>
       </c>
@@ -2002,8 +2110,11 @@
       <c r="G37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H37">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>3</v>
       </c>
@@ -2025,8 +2136,11 @@
       <c r="G38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H38">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -2048,8 +2162,11 @@
       <c r="G39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H39">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>3</v>
       </c>
@@ -2071,8 +2188,11 @@
       <c r="G40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H40">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -2094,8 +2214,11 @@
       <c r="G41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H41">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -2117,8 +2240,11 @@
       <c r="G42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H42">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>3</v>
       </c>
@@ -2140,8 +2266,11 @@
       <c r="G43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H43">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>40</v>
       </c>
@@ -2163,8 +2292,11 @@
       <c r="G44">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H44">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>3</v>
       </c>
@@ -2186,8 +2318,11 @@
       <c r="G45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H45">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -2209,8 +2344,11 @@
       <c r="G46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H46">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>3</v>
       </c>
@@ -2232,8 +2370,11 @@
       <c r="G47">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H47">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>3</v>
       </c>
@@ -2255,8 +2396,11 @@
       <c r="G48">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H48">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -2278,8 +2422,11 @@
       <c r="G49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H49">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>3</v>
       </c>
@@ -2301,8 +2448,11 @@
       <c r="G50">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H50">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>3</v>
       </c>
@@ -2324,8 +2474,11 @@
       <c r="G51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H51">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>3</v>
       </c>
@@ -2347,8 +2500,11 @@
       <c r="G52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H52">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>3</v>
       </c>
@@ -2370,8 +2526,11 @@
       <c r="G53">
         <v>1</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H53">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>3</v>
       </c>
@@ -2393,8 +2552,11 @@
       <c r="G54">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H54">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>3</v>
       </c>
@@ -2416,8 +2578,11 @@
       <c r="G55">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H55">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>3</v>
       </c>
@@ -2439,8 +2604,11 @@
       <c r="G56">
         <v>1</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H56">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>3</v>
       </c>
@@ -2462,8 +2630,11 @@
       <c r="G57">
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H57">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>3</v>
       </c>
@@ -2485,8 +2656,11 @@
       <c r="G58">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H58">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>3</v>
       </c>
@@ -2508,8 +2682,11 @@
       <c r="G59">
         <v>1</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H59">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>40</v>
       </c>
@@ -2531,8 +2708,11 @@
       <c r="G60">
         <v>1</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H60">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>40</v>
       </c>
@@ -2554,8 +2734,11 @@
       <c r="G61">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H61">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>3</v>
       </c>
@@ -2577,8 +2760,11 @@
       <c r="G62">
         <v>1</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H62">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>3</v>
       </c>
@@ -2600,8 +2786,11 @@
       <c r="G63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H63">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>3</v>
       </c>
@@ -2623,8 +2812,11 @@
       <c r="G64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H64">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>3</v>
       </c>
@@ -2646,8 +2838,11 @@
       <c r="G65">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H65">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>3</v>
       </c>
@@ -2669,8 +2864,11 @@
       <c r="G66">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H66">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>3</v>
       </c>
@@ -2692,8 +2890,11 @@
       <c r="G67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H67">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>3</v>
       </c>
@@ -2715,8 +2916,11 @@
       <c r="G68">
         <v>0.3</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H68">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>3</v>
       </c>
@@ -2736,6 +2940,9 @@
         <v>0.2</v>
       </c>
       <c r="G69">
+        <v>0.3</v>
+      </c>
+      <c r="H69">
         <v>0.3</v>
       </c>
     </row>
@@ -2746,6 +2953,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="93b6acfe-855d-4bce-87e8-8301fe2e15c6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002CCAD73C6C0AE44F90B1789BF56DE2C9" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7b9dae6affa01c469eabe825fd34801d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="93b6acfe-855d-4bce-87e8-8301fe2e15c6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9cd683c8972a97d9da195e07efd4ebfc" ns3:_="">
     <xsd:import namespace="93b6acfe-855d-4bce-87e8-8301fe2e15c6"/>
@@ -2895,24 +3119,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3404FE83-9920-4C23-968A-2F9E70DCE3C6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="93b6acfe-855d-4bce-87e8-8301fe2e15c6"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="93b6acfe-855d-4bce-87e8-8301fe2e15c6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C935EC73-C13B-4C3B-B5EC-977831D6D4E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{952EA37B-F1EC-404E-BD4F-10BB1041C0F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2928,28 +3159,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C935EC73-C13B-4C3B-B5EC-977831D6D4E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3404FE83-9920-4C23-968A-2F9E70DCE3C6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="93b6acfe-855d-4bce-87e8-8301fe2e15c6"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update the feeding and dispersal guild information
</commit_message>
<xml_diff>
--- a/data/topID feeding guild.xlsx
+++ b/data/topID feeding guild.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\osawe\Documents\Git\cc-urbanization\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78ED513-8519-4154-84DF-283C792FB51A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F7F002-FE95-493A-A123-6427F5BD3DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22335" yWindow="3480" windowWidth="23865" windowHeight="17655" xr2:uid="{49CD93DB-F6D1-459A-A250-6E9A2941DB32}"/>
+    <workbookView xWindow="5775" yWindow="2910" windowWidth="23865" windowHeight="17655" activeTab="1" xr2:uid="{49CD93DB-F6D1-459A-A250-6E9A2941DB32}"/>
   </bookViews>
   <sheets>
     <sheet name="topID" sheetId="1" r:id="rId1"/>
+    <sheet name="topID2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="133">
   <si>
     <t>Rank</t>
   </si>
@@ -284,6 +285,141 @@
   </si>
   <si>
     <t>Dispersal_Flight</t>
+  </si>
+  <si>
+    <t>Myrmica</t>
+  </si>
+  <si>
+    <t>Lasius</t>
+  </si>
+  <si>
+    <t>Hyphantria</t>
+  </si>
+  <si>
+    <t>Epimecis</t>
+  </si>
+  <si>
+    <t>Pyreferra</t>
+  </si>
+  <si>
+    <t>Hypagyrtis</t>
+  </si>
+  <si>
+    <t>Lymantriinae</t>
+  </si>
+  <si>
+    <t>Anisota</t>
+  </si>
+  <si>
+    <t>Amphipyra</t>
+  </si>
+  <si>
+    <t>Limacodinae</t>
+  </si>
+  <si>
+    <t>Malacosoma</t>
+  </si>
+  <si>
+    <t>Colocasia</t>
+  </si>
+  <si>
+    <t>Photuris</t>
+  </si>
+  <si>
+    <t>Pseudocneorhinus</t>
+  </si>
+  <si>
+    <t>Phyllobius</t>
+  </si>
+  <si>
+    <t>Cryptocephalus</t>
+  </si>
+  <si>
+    <t>Odontopus</t>
+  </si>
+  <si>
+    <t>Demotina</t>
+  </si>
+  <si>
+    <t>Anyphaena</t>
+  </si>
+  <si>
+    <t>Enoplognatha</t>
+  </si>
+  <si>
+    <t>Mangora</t>
+  </si>
+  <si>
+    <t>Paraphidippus</t>
+  </si>
+  <si>
+    <t>Gyponana</t>
+  </si>
+  <si>
+    <t>Platycotis</t>
+  </si>
+  <si>
+    <t>Typhlocybinae</t>
+  </si>
+  <si>
+    <t>Orientus</t>
+  </si>
+  <si>
+    <t>Clastoptera</t>
+  </si>
+  <si>
+    <t>Japananus</t>
+  </si>
+  <si>
+    <t>Pselliopus</t>
+  </si>
+  <si>
+    <t>Halyomorpha</t>
+  </si>
+  <si>
+    <t>Podisus</t>
+  </si>
+  <si>
+    <t>Emesinae</t>
+  </si>
+  <si>
+    <t>Brochymena</t>
+  </si>
+  <si>
+    <t>Sciapodinae</t>
+  </si>
+  <si>
+    <t>Rhagio</t>
+  </si>
+  <si>
+    <t>Delphinia</t>
+  </si>
+  <si>
+    <t>Macrocera</t>
+  </si>
+  <si>
+    <t>Toxomerus</t>
+  </si>
+  <si>
+    <t>Chironominae</t>
+  </si>
+  <si>
+    <t>Macrodiplosis</t>
+  </si>
+  <si>
+    <t>Meconema</t>
+  </si>
+  <si>
+    <t>Feeding_method</t>
+  </si>
+  <si>
+    <t>chewers</t>
+  </si>
+  <si>
+    <t>suckers</t>
+  </si>
+  <si>
+    <t>sucker</t>
   </si>
 </sst>
 </file>
@@ -2952,24 +3088,2412 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="93b6acfe-855d-4bce-87e8-8301fe2e15c6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF58ED1A-8785-4D70-946C-A61D2E4E6AA3}">
+  <dimension ref="A1:G110"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>0.5</v>
+      </c>
+      <c r="E2">
+        <v>0.5</v>
+      </c>
+      <c r="F2">
+        <v>0.5</v>
+      </c>
+      <c r="G2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5">
+        <v>0.5</v>
+      </c>
+      <c r="E5">
+        <v>0.5</v>
+      </c>
+      <c r="F5">
+        <v>0.5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0.5</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0.5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0.5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0.5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0.5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0.5</v>
+      </c>
+      <c r="G12" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0.5</v>
+      </c>
+      <c r="G13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0.5</v>
+      </c>
+      <c r="G14" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0.5</v>
+      </c>
+      <c r="G15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0.5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0.5</v>
+      </c>
+      <c r="G17" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0.5</v>
+      </c>
+      <c r="G18" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0.5</v>
+      </c>
+      <c r="G19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0.5</v>
+      </c>
+      <c r="G20" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0.5</v>
+      </c>
+      <c r="G21" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0.5</v>
+      </c>
+      <c r="G22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0.5</v>
+      </c>
+      <c r="G23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0.5</v>
+      </c>
+      <c r="G25" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0.5</v>
+      </c>
+      <c r="G26" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0.5</v>
+      </c>
+      <c r="G28" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>0.5</v>
+      </c>
+      <c r="G32" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>100</v>
+      </c>
+      <c r="C33" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33">
+        <v>0</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0.5</v>
+      </c>
+      <c r="G34" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
+        <v>102</v>
+      </c>
+      <c r="C35" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0.5</v>
+      </c>
+      <c r="G35" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36">
+        <v>0</v>
+      </c>
+      <c r="F36">
+        <v>0.5</v>
+      </c>
+      <c r="G36" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" t="s">
+        <v>104</v>
+      </c>
+      <c r="C37" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0.5</v>
+      </c>
+      <c r="G37" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>3</v>
+      </c>
+      <c r="B38" t="s">
+        <v>105</v>
+      </c>
+      <c r="C38" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>0.5</v>
+      </c>
+      <c r="G38" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>3</v>
+      </c>
+      <c r="B39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39" t="s">
+        <v>28</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>3</v>
+      </c>
+      <c r="B40" t="s">
+        <v>29</v>
+      </c>
+      <c r="C40" t="s">
+        <v>28</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>3</v>
+      </c>
+      <c r="B41" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41" t="s">
+        <v>28</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>3</v>
+      </c>
+      <c r="B42" t="s">
+        <v>31</v>
+      </c>
+      <c r="C42" t="s">
+        <v>28</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>3</v>
+      </c>
+      <c r="B43" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43" t="s">
+        <v>28</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>3</v>
+      </c>
+      <c r="B44" t="s">
+        <v>32</v>
+      </c>
+      <c r="C44" t="s">
+        <v>28</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" t="s">
+        <v>28</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>3</v>
+      </c>
+      <c r="B46" t="s">
+        <v>36</v>
+      </c>
+      <c r="C46" t="s">
+        <v>28</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>3</v>
+      </c>
+      <c r="B47" t="s">
+        <v>37</v>
+      </c>
+      <c r="C47" t="s">
+        <v>28</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>3</v>
+      </c>
+      <c r="B48" t="s">
+        <v>35</v>
+      </c>
+      <c r="C48" t="s">
+        <v>28</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>3</v>
+      </c>
+      <c r="B49" t="s">
+        <v>38</v>
+      </c>
+      <c r="C49" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B50" t="s">
+        <v>41</v>
+      </c>
+      <c r="C50" t="s">
+        <v>28</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>3</v>
+      </c>
+      <c r="B51" t="s">
+        <v>39</v>
+      </c>
+      <c r="C51" t="s">
+        <v>28</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>3</v>
+      </c>
+      <c r="B52" t="s">
+        <v>42</v>
+      </c>
+      <c r="C52" t="s">
+        <v>28</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>3</v>
+      </c>
+      <c r="B53" t="s">
+        <v>43</v>
+      </c>
+      <c r="C53" t="s">
+        <v>28</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>3</v>
+      </c>
+      <c r="B54" t="s">
+        <v>44</v>
+      </c>
+      <c r="C54" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+      <c r="F54">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>3</v>
+      </c>
+      <c r="B55" t="s">
+        <v>106</v>
+      </c>
+      <c r="C55" t="s">
+        <v>28</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>3</v>
+      </c>
+      <c r="B56" t="s">
+        <v>107</v>
+      </c>
+      <c r="C56" t="s">
+        <v>28</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>3</v>
+      </c>
+      <c r="B57" t="s">
+        <v>108</v>
+      </c>
+      <c r="C57" t="s">
+        <v>28</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+      <c r="F57">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>3</v>
+      </c>
+      <c r="B58" t="s">
+        <v>109</v>
+      </c>
+      <c r="C58" t="s">
+        <v>28</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>3</v>
+      </c>
+      <c r="B59" t="s">
+        <v>45</v>
+      </c>
+      <c r="C59" t="s">
+        <v>46</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>1</v>
+      </c>
+      <c r="G59" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>3</v>
+      </c>
+      <c r="B60" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" t="s">
+        <v>46</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>1</v>
+      </c>
+      <c r="G60" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>3</v>
+      </c>
+      <c r="B61" t="s">
+        <v>48</v>
+      </c>
+      <c r="C61" t="s">
+        <v>46</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>1</v>
+      </c>
+      <c r="G61" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>3</v>
+      </c>
+      <c r="B62" t="s">
+        <v>49</v>
+      </c>
+      <c r="C62" t="s">
+        <v>46</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+      <c r="G62" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>3</v>
+      </c>
+      <c r="B63" t="s">
+        <v>50</v>
+      </c>
+      <c r="C63" t="s">
+        <v>46</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>40</v>
+      </c>
+      <c r="B64" t="s">
+        <v>51</v>
+      </c>
+      <c r="C64" t="s">
+        <v>46</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>1</v>
+      </c>
+      <c r="G64" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" t="s">
+        <v>52</v>
+      </c>
+      <c r="C65" t="s">
+        <v>46</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>1</v>
+      </c>
+      <c r="G65" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>40</v>
+      </c>
+      <c r="B66" t="s">
+        <v>53</v>
+      </c>
+      <c r="C66" t="s">
+        <v>46</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>1</v>
+      </c>
+      <c r="G66" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>3</v>
+      </c>
+      <c r="B67" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" t="s">
+        <v>46</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>1</v>
+      </c>
+      <c r="G67" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>3</v>
+      </c>
+      <c r="B68" t="s">
+        <v>55</v>
+      </c>
+      <c r="C68" t="s">
+        <v>46</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>1</v>
+      </c>
+      <c r="G68" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>3</v>
+      </c>
+      <c r="B69" t="s">
+        <v>110</v>
+      </c>
+      <c r="C69" t="s">
+        <v>46</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+      <c r="G69" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>3</v>
+      </c>
+      <c r="B70" t="s">
+        <v>111</v>
+      </c>
+      <c r="C70" t="s">
+        <v>46</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>1</v>
+      </c>
+      <c r="G70" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>25</v>
+      </c>
+      <c r="B71" t="s">
+        <v>112</v>
+      </c>
+      <c r="C71" t="s">
+        <v>46</v>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+      <c r="E71">
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>1</v>
+      </c>
+      <c r="G71" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>3</v>
+      </c>
+      <c r="B72" t="s">
+        <v>113</v>
+      </c>
+      <c r="C72" t="s">
+        <v>46</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>1</v>
+      </c>
+      <c r="G72" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>3</v>
+      </c>
+      <c r="B73" t="s">
+        <v>114</v>
+      </c>
+      <c r="C73" t="s">
+        <v>46</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+      <c r="E73">
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>1</v>
+      </c>
+      <c r="G73" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>3</v>
+      </c>
+      <c r="B74" t="s">
+        <v>115</v>
+      </c>
+      <c r="C74" t="s">
+        <v>46</v>
+      </c>
+      <c r="D74">
+        <v>1</v>
+      </c>
+      <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>1</v>
+      </c>
+      <c r="G74" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>3</v>
+      </c>
+      <c r="B75" t="s">
+        <v>56</v>
+      </c>
+      <c r="C75" t="s">
+        <v>57</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+      <c r="E75">
+        <v>1</v>
+      </c>
+      <c r="F75">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>3</v>
+      </c>
+      <c r="B76" t="s">
+        <v>58</v>
+      </c>
+      <c r="C76" t="s">
+        <v>57</v>
+      </c>
+      <c r="D76">
+        <v>0.5</v>
+      </c>
+      <c r="E76">
+        <v>0.5</v>
+      </c>
+      <c r="F76">
+        <v>0.5</v>
+      </c>
+      <c r="G76" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>3</v>
+      </c>
+      <c r="B77" t="s">
+        <v>59</v>
+      </c>
+      <c r="C77" t="s">
+        <v>57</v>
+      </c>
+      <c r="D77">
+        <v>0.5</v>
+      </c>
+      <c r="E77">
+        <v>0.5</v>
+      </c>
+      <c r="F77">
+        <v>0.5</v>
+      </c>
+      <c r="G77" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>3</v>
+      </c>
+      <c r="B78" t="s">
+        <v>60</v>
+      </c>
+      <c r="C78" t="s">
+        <v>57</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78">
+        <v>1</v>
+      </c>
+      <c r="F78">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>3</v>
+      </c>
+      <c r="B79" t="s">
+        <v>61</v>
+      </c>
+      <c r="C79" t="s">
+        <v>57</v>
+      </c>
+      <c r="D79">
+        <v>1</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>0.5</v>
+      </c>
+      <c r="G79" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>3</v>
+      </c>
+      <c r="B80" t="s">
+        <v>62</v>
+      </c>
+      <c r="C80" t="s">
+        <v>57</v>
+      </c>
+      <c r="D80">
+        <v>1</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>0.5</v>
+      </c>
+      <c r="G80" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>3</v>
+      </c>
+      <c r="B81" t="s">
+        <v>63</v>
+      </c>
+      <c r="C81" t="s">
+        <v>57</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>3</v>
+      </c>
+      <c r="B82" t="s">
+        <v>64</v>
+      </c>
+      <c r="C82" t="s">
+        <v>57</v>
+      </c>
+      <c r="D82">
+        <v>1</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>0.5</v>
+      </c>
+      <c r="G82" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>3</v>
+      </c>
+      <c r="B83" t="s">
+        <v>65</v>
+      </c>
+      <c r="C83" t="s">
+        <v>57</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>0.5</v>
+      </c>
+      <c r="G83" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>3</v>
+      </c>
+      <c r="B84" t="s">
+        <v>116</v>
+      </c>
+      <c r="C84" t="s">
+        <v>57</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>3</v>
+      </c>
+      <c r="B85" t="s">
+        <v>117</v>
+      </c>
+      <c r="C85" t="s">
+        <v>57</v>
+      </c>
+      <c r="D85">
+        <v>1</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>0.5</v>
+      </c>
+      <c r="G85" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>3</v>
+      </c>
+      <c r="B86" t="s">
+        <v>118</v>
+      </c>
+      <c r="C86" t="s">
+        <v>57</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>25</v>
+      </c>
+      <c r="B87" t="s">
+        <v>119</v>
+      </c>
+      <c r="C87" t="s">
+        <v>57</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>1</v>
+      </c>
+      <c r="F87">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>3</v>
+      </c>
+      <c r="B88" t="s">
+        <v>120</v>
+      </c>
+      <c r="C88" t="s">
+        <v>57</v>
+      </c>
+      <c r="D88">
+        <v>0.5</v>
+      </c>
+      <c r="E88">
+        <v>0.5</v>
+      </c>
+      <c r="F88">
+        <v>0.5</v>
+      </c>
+      <c r="G88" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>3</v>
+      </c>
+      <c r="B89" t="s">
+        <v>66</v>
+      </c>
+      <c r="C89" t="s">
+        <v>67</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>1</v>
+      </c>
+      <c r="F89">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>3</v>
+      </c>
+      <c r="B90" t="s">
+        <v>68</v>
+      </c>
+      <c r="C90" t="s">
+        <v>67</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>1</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>3</v>
+      </c>
+      <c r="B91" t="s">
+        <v>69</v>
+      </c>
+      <c r="C91" t="s">
+        <v>67</v>
+      </c>
+      <c r="D91">
+        <v>0.5</v>
+      </c>
+      <c r="E91">
+        <v>0.5</v>
+      </c>
+      <c r="F91">
+        <v>1</v>
+      </c>
+      <c r="G91" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>3</v>
+      </c>
+      <c r="B92" t="s">
+        <v>70</v>
+      </c>
+      <c r="C92" t="s">
+        <v>67</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>1</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>40</v>
+      </c>
+      <c r="B93" t="s">
+        <v>71</v>
+      </c>
+      <c r="C93" t="s">
+        <v>67</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>1</v>
+      </c>
+      <c r="F93">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>40</v>
+      </c>
+      <c r="B94" t="s">
+        <v>72</v>
+      </c>
+      <c r="C94" t="s">
+        <v>67</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
+        <v>1</v>
+      </c>
+      <c r="F94">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>3</v>
+      </c>
+      <c r="B95" t="s">
+        <v>73</v>
+      </c>
+      <c r="C95" t="s">
+        <v>67</v>
+      </c>
+      <c r="D95">
+        <v>0</v>
+      </c>
+      <c r="E95">
+        <v>1</v>
+      </c>
+      <c r="F95">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>3</v>
+      </c>
+      <c r="B96" t="s">
+        <v>74</v>
+      </c>
+      <c r="C96" t="s">
+        <v>67</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96">
+        <v>1</v>
+      </c>
+      <c r="F96">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>25</v>
+      </c>
+      <c r="B97" t="s">
+        <v>121</v>
+      </c>
+      <c r="C97" t="s">
+        <v>67</v>
+      </c>
+      <c r="D97">
+        <v>0</v>
+      </c>
+      <c r="E97">
+        <v>1</v>
+      </c>
+      <c r="F97">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>3</v>
+      </c>
+      <c r="B98" t="s">
+        <v>122</v>
+      </c>
+      <c r="C98" t="s">
+        <v>67</v>
+      </c>
+      <c r="D98">
+        <v>0</v>
+      </c>
+      <c r="E98">
+        <v>1</v>
+      </c>
+      <c r="F98">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>3</v>
+      </c>
+      <c r="B99" t="s">
+        <v>123</v>
+      </c>
+      <c r="C99" t="s">
+        <v>67</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>1</v>
+      </c>
+      <c r="F99">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>3</v>
+      </c>
+      <c r="B100" t="s">
+        <v>124</v>
+      </c>
+      <c r="C100" t="s">
+        <v>67</v>
+      </c>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="E100">
+        <v>1</v>
+      </c>
+      <c r="F100">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>3</v>
+      </c>
+      <c r="B101" t="s">
+        <v>125</v>
+      </c>
+      <c r="C101" t="s">
+        <v>67</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101">
+        <v>0</v>
+      </c>
+      <c r="F101">
+        <v>1</v>
+      </c>
+      <c r="G101" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>25</v>
+      </c>
+      <c r="B102" t="s">
+        <v>126</v>
+      </c>
+      <c r="C102" t="s">
+        <v>67</v>
+      </c>
+      <c r="D102">
+        <v>1</v>
+      </c>
+      <c r="E102">
+        <v>0</v>
+      </c>
+      <c r="F102">
+        <v>1</v>
+      </c>
+      <c r="G102" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>3</v>
+      </c>
+      <c r="B103" t="s">
+        <v>127</v>
+      </c>
+      <c r="C103" t="s">
+        <v>67</v>
+      </c>
+      <c r="D103">
+        <v>1</v>
+      </c>
+      <c r="E103">
+        <v>0</v>
+      </c>
+      <c r="F103">
+        <v>0.5</v>
+      </c>
+      <c r="G103" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>3</v>
+      </c>
+      <c r="B104" t="s">
+        <v>75</v>
+      </c>
+      <c r="C104" t="s">
+        <v>76</v>
+      </c>
+      <c r="D104">
+        <v>1</v>
+      </c>
+      <c r="E104">
+        <v>0</v>
+      </c>
+      <c r="F104">
+        <v>1</v>
+      </c>
+      <c r="G104" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>3</v>
+      </c>
+      <c r="B105" t="s">
+        <v>77</v>
+      </c>
+      <c r="C105" t="s">
+        <v>76</v>
+      </c>
+      <c r="D105">
+        <v>1</v>
+      </c>
+      <c r="E105">
+        <v>0</v>
+      </c>
+      <c r="F105">
+        <v>0.5</v>
+      </c>
+      <c r="G105" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>3</v>
+      </c>
+      <c r="B106" t="s">
+        <v>78</v>
+      </c>
+      <c r="C106" t="s">
+        <v>76</v>
+      </c>
+      <c r="D106">
+        <v>1</v>
+      </c>
+      <c r="E106">
+        <v>0</v>
+      </c>
+      <c r="F106">
+        <v>0.5</v>
+      </c>
+      <c r="G106" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>3</v>
+      </c>
+      <c r="B107" t="s">
+        <v>79</v>
+      </c>
+      <c r="C107" t="s">
+        <v>76</v>
+      </c>
+      <c r="D107">
+        <v>1</v>
+      </c>
+      <c r="E107">
+        <v>0</v>
+      </c>
+      <c r="F107">
+        <v>0.5</v>
+      </c>
+      <c r="G107" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>3</v>
+      </c>
+      <c r="B108" t="s">
+        <v>128</v>
+      </c>
+      <c r="C108" t="s">
+        <v>76</v>
+      </c>
+      <c r="D108">
+        <v>1</v>
+      </c>
+      <c r="E108">
+        <v>0</v>
+      </c>
+      <c r="F108">
+        <v>0.5</v>
+      </c>
+      <c r="G108" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>3</v>
+      </c>
+      <c r="B109" t="s">
+        <v>80</v>
+      </c>
+      <c r="C109" t="s">
+        <v>81</v>
+      </c>
+      <c r="D109">
+        <v>0</v>
+      </c>
+      <c r="E109">
+        <v>0.5</v>
+      </c>
+      <c r="F109">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>3</v>
+      </c>
+      <c r="B110" t="s">
+        <v>82</v>
+      </c>
+      <c r="C110" t="s">
+        <v>81</v>
+      </c>
+      <c r="D110">
+        <v>0</v>
+      </c>
+      <c r="E110">
+        <v>0.5</v>
+      </c>
+      <c r="F110">
+        <v>0.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002CCAD73C6C0AE44F90B1789BF56DE2C9" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7b9dae6affa01c469eabe825fd34801d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="93b6acfe-855d-4bce-87e8-8301fe2e15c6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9cd683c8972a97d9da195e07efd4ebfc" ns3:_="">
     <xsd:import namespace="93b6acfe-855d-4bce-87e8-8301fe2e15c6"/>
@@ -3119,7 +5643,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="93b6acfe-855d-4bce-87e8-8301fe2e15c6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{952EA37B-F1EC-404E-BD4F-10BB1041C0F3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="93b6acfe-855d-4bce-87e8-8301fe2e15c6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3404FE83-9920-4C23-968A-2F9E70DCE3C6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -3135,28 +5694,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C935EC73-C13B-4C3B-B5EC-977831D6D4E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{952EA37B-F1EC-404E-BD4F-10BB1041C0F3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="93b6acfe-855d-4bce-87e8-8301fe2e15c6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>